<commit_message>
Add Events tag, GP Sessions post, retag Real Estate Gala
</commit_message>
<xml_diff>
--- a/Links.xlsx
+++ b/Links.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="355" uniqueCount="186">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="359" uniqueCount="188">
   <si>
     <t>title</t>
   </si>
@@ -158,13 +158,16 @@
     <t>The Real Estate Gala teaser</t>
   </si>
   <si>
+    <t>Events</t>
+  </si>
+  <si>
     <t>https://youtube.com/shorts/CtIohUSPn2Q?feature=share</t>
   </si>
   <si>
     <t>The Real Estate Gala countdown- 1 day left</t>
   </si>
   <si>
-    <t>AI, Brand</t>
+    <t>AI, Events</t>
   </si>
   <si>
     <t>https://youtu.be/uUCTqt_5Qvc</t>
@@ -458,6 +461,12 @@
     <t>https://www.linkedin.com/feed/update/urn:li:activity:7312836217748774915</t>
   </si>
   <si>
+    <t>GP Sessions fireside discussion</t>
+  </si>
+  <si>
+    <t>https://www.linkedin.com/feed/update/urn:li:activity:7460689339107422208</t>
+  </si>
+  <si>
     <t>Theme</t>
   </si>
   <si>
@@ -608,9 +617,6 @@
       </rPr>
       <t>Agora growth awards teaser</t>
     </r>
-  </si>
-  <si>
-    <t>Events</t>
   </si>
   <si>
     <r>
@@ -1978,13 +1984,13 @@
         <v>47</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>23</v>
+        <v>48</v>
       </c>
       <c r="C15" s="3" t="s">
         <v>8</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="E15" s="3" t="s">
         <v>10</v>
@@ -2016,16 +2022,16 @@
     </row>
     <row r="16">
       <c r="A16" s="3" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C16" s="3" t="s">
         <v>8</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="E16" s="3" t="s">
         <v>18</v>
@@ -2052,16 +2058,16 @@
     </row>
     <row r="17">
       <c r="A17" s="3" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C17" s="3" t="s">
         <v>8</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="E17" s="3" t="s">
         <v>18</v>
@@ -2069,7 +2075,7 @@
       <c r="F17" s="2"/>
       <c r="G17" s="2"/>
       <c r="H17" s="6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="I17" s="2"/>
       <c r="J17" s="2"/>
@@ -2091,16 +2097,16 @@
     </row>
     <row r="18">
       <c r="A18" s="3" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C18" s="3" t="s">
         <v>8</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="E18" s="3" t="s">
         <v>18</v>
@@ -2128,16 +2134,16 @@
     </row>
     <row r="19">
       <c r="A19" s="3" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C19" s="3" t="s">
         <v>8</v>
       </c>
       <c r="D19" s="4" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="E19" s="3" t="s">
         <v>18</v>
@@ -2165,16 +2171,16 @@
     </row>
     <row r="20">
       <c r="A20" s="3" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C20" s="3" t="s">
         <v>8</v>
       </c>
       <c r="D20" s="4" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="E20" s="3" t="s">
         <v>18</v>
@@ -2202,16 +2208,16 @@
     </row>
     <row r="21">
       <c r="A21" s="3" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C21" s="3" t="s">
         <v>8</v>
       </c>
       <c r="D21" s="4" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="E21" s="3" t="s">
         <v>18</v>
@@ -2239,16 +2245,16 @@
     </row>
     <row r="22">
       <c r="A22" s="3" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C22" s="3" t="s">
         <v>8</v>
       </c>
       <c r="D22" s="4" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="E22" s="3" t="s">
         <v>18</v>
@@ -2279,14 +2285,14 @@
         <v>15</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C23" s="3" t="s">
         <v>8</v>
       </c>
       <c r="D23" s="2"/>
       <c r="E23" s="3" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="F23" s="3" t="s">
         <v>11</v>
@@ -2313,19 +2319,19 @@
     </row>
     <row r="24">
       <c r="A24" s="3" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B24" s="6" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="C24" s="3" t="s">
         <v>8</v>
       </c>
       <c r="D24" s="4" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="E24" s="3" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="F24" s="2"/>
       <c r="G24" s="2"/>
@@ -2350,7 +2356,7 @@
     </row>
     <row r="25">
       <c r="A25" s="3" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B25" s="6" t="s">
         <v>23</v>
@@ -2359,10 +2365,10 @@
         <v>8</v>
       </c>
       <c r="D25" s="4" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="E25" s="3" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="F25" s="3" t="s">
         <v>11</v>
@@ -2389,19 +2395,19 @@
     </row>
     <row r="26">
       <c r="A26" s="3" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C26" s="3" t="s">
         <v>8</v>
       </c>
       <c r="D26" s="4" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="E26" s="3" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="F26" s="3" t="s">
         <v>11</v>
@@ -2428,19 +2434,19 @@
     </row>
     <row r="27">
       <c r="A27" s="3" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="B27" s="6" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="C27" s="3" t="s">
         <v>8</v>
       </c>
       <c r="D27" s="4" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="E27" s="3" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="F27" s="2"/>
       <c r="G27" s="2"/>
@@ -2465,7 +2471,7 @@
     </row>
     <row r="28">
       <c r="A28" s="3" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="B28" s="6" t="s">
         <v>23</v>
@@ -2474,10 +2480,10 @@
         <v>8</v>
       </c>
       <c r="D28" s="4" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="E28" s="3" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="F28" s="2"/>
       <c r="G28" s="2"/>
@@ -2502,7 +2508,7 @@
     </row>
     <row r="29">
       <c r="A29" s="3" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="B29" s="3" t="s">
         <v>7</v>
@@ -2511,7 +2517,7 @@
         <v>8</v>
       </c>
       <c r="D29" s="4" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="E29" s="3" t="s">
         <v>10</v>
@@ -2539,19 +2545,19 @@
     </row>
     <row r="30">
       <c r="A30" s="3" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="B30" s="6" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="C30" s="3" t="s">
         <v>8</v>
       </c>
       <c r="D30" s="4" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="E30" s="3" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="F30" s="3" t="s">
         <v>11</v>
@@ -2578,19 +2584,19 @@
     </row>
     <row r="31">
       <c r="A31" s="3" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="B31" s="6" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="C31" s="3" t="s">
         <v>8</v>
       </c>
       <c r="D31" s="4" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="E31" s="3" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="F31" s="3" t="s">
         <v>11</v>
@@ -2617,19 +2623,19 @@
     </row>
     <row r="32">
       <c r="A32" s="3" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="B32" s="6" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="C32" s="3" t="s">
         <v>8</v>
       </c>
       <c r="D32" s="4" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="E32" s="3" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="F32" s="3" t="s">
         <v>11</v>
@@ -2656,19 +2662,19 @@
     </row>
     <row r="33">
       <c r="A33" s="3" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="B33" s="6" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="C33" s="3" t="s">
         <v>8</v>
       </c>
       <c r="D33" s="4" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="E33" s="3" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="F33" s="3" t="s">
         <v>11</v>
@@ -2695,19 +2701,19 @@
     </row>
     <row r="34">
       <c r="A34" s="3" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="B34" s="6" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="C34" s="3" t="s">
         <v>8</v>
       </c>
       <c r="D34" s="4" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="E34" s="3" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="F34" s="3" t="s">
         <v>11</v>
@@ -2734,19 +2740,19 @@
     </row>
     <row r="35">
       <c r="A35" s="3" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="B35" s="6" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="C35" s="3" t="s">
         <v>8</v>
       </c>
       <c r="D35" s="4" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="E35" s="3" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="F35" s="3" t="s">
         <v>11</v>
@@ -2773,19 +2779,19 @@
     </row>
     <row r="36">
       <c r="A36" s="3" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="B36" s="6" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="C36" s="3" t="s">
         <v>8</v>
       </c>
       <c r="D36" s="4" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="E36" s="3" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="F36" s="2"/>
       <c r="G36" s="2"/>
@@ -2810,19 +2816,19 @@
     </row>
     <row r="37">
       <c r="A37" s="3" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="B37" s="6" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="C37" s="3" t="s">
         <v>8</v>
       </c>
       <c r="D37" s="5" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="E37" s="3" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="F37" s="2"/>
       <c r="G37" s="2"/>
@@ -2847,19 +2853,19 @@
     </row>
     <row r="38">
       <c r="A38" s="3" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B38" s="6" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="C38" s="3" t="s">
         <v>8</v>
       </c>
       <c r="D38" s="4" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="E38" s="3" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="F38" s="2"/>
       <c r="G38" s="2"/>
@@ -2884,19 +2890,19 @@
     </row>
     <row r="39">
       <c r="A39" s="3" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="B39" s="6" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="C39" s="3" t="s">
         <v>8</v>
       </c>
       <c r="D39" s="4" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="E39" s="3" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="F39" s="2"/>
       <c r="G39" s="2"/>
@@ -2921,19 +2927,19 @@
     </row>
     <row r="40">
       <c r="A40" s="3" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="B40" s="6" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="C40" s="3" t="s">
         <v>8</v>
       </c>
       <c r="D40" s="4" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="E40" s="3" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="F40" s="2"/>
       <c r="G40" s="2"/>
@@ -2958,19 +2964,19 @@
     </row>
     <row r="41">
       <c r="A41" s="3" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="B41" s="6" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="C41" s="3" t="s">
         <v>8</v>
       </c>
       <c r="D41" s="4" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="E41" s="3" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="F41" s="2"/>
       <c r="G41" s="2"/>
@@ -2995,16 +3001,16 @@
     </row>
     <row r="42">
       <c r="A42" s="7" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="B42" s="6" t="s">
         <v>46</v>
       </c>
       <c r="C42" s="6" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="D42" s="4" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="E42" s="2"/>
       <c r="F42" s="2"/>
@@ -3030,16 +3036,16 @@
     </row>
     <row r="43">
       <c r="A43" s="7" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B43" s="6" t="s">
         <v>46</v>
       </c>
       <c r="C43" s="6" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="D43" s="4" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="E43" s="2"/>
       <c r="F43" s="2"/>
@@ -3065,16 +3071,16 @@
     </row>
     <row r="44">
       <c r="A44" s="7" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="B44" s="6" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="C44" s="6" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="D44" s="4" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="E44" s="2"/>
       <c r="F44" s="2"/>
@@ -3100,16 +3106,16 @@
     </row>
     <row r="45">
       <c r="A45" s="7" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="B45" s="6" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="C45" s="6" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="D45" s="4" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="E45" s="2"/>
       <c r="F45" s="2"/>
@@ -3135,16 +3141,16 @@
     </row>
     <row r="46">
       <c r="A46" s="7" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="B46" s="6" t="s">
         <v>46</v>
       </c>
       <c r="C46" s="6" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="D46" s="4" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="E46" s="2"/>
       <c r="F46" s="2"/>
@@ -3170,16 +3176,16 @@
     </row>
     <row r="47">
       <c r="A47" s="7" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="B47" s="6" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="C47" s="6" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="D47" s="4" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="E47" s="2"/>
       <c r="F47" s="2"/>
@@ -3205,16 +3211,16 @@
     </row>
     <row r="48">
       <c r="A48" s="7" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="B48" s="6" t="s">
         <v>46</v>
       </c>
       <c r="C48" s="6" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="D48" s="4" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="E48" s="2"/>
       <c r="F48" s="2"/>
@@ -3240,16 +3246,16 @@
     </row>
     <row r="49">
       <c r="A49" s="7" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="B49" s="6" t="s">
         <v>46</v>
       </c>
       <c r="C49" s="6" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="D49" s="4" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="E49" s="2"/>
       <c r="F49" s="2"/>
@@ -3275,16 +3281,16 @@
     </row>
     <row r="50">
       <c r="A50" s="7" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="B50" s="6" t="s">
         <v>46</v>
       </c>
       <c r="C50" s="6" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="D50" s="4" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="E50" s="2"/>
       <c r="F50" s="2"/>
@@ -3310,16 +3316,16 @@
     </row>
     <row r="51">
       <c r="A51" s="7" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="B51" s="6" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="C51" s="6" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="D51" s="4" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="E51" s="2"/>
       <c r="F51" s="2"/>
@@ -3345,16 +3351,16 @@
     </row>
     <row r="52">
       <c r="A52" s="7" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="B52" s="6" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="C52" s="6" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="D52" s="4" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="E52" s="2"/>
       <c r="F52" s="2"/>
@@ -3380,16 +3386,16 @@
     </row>
     <row r="53">
       <c r="A53" s="7" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="B53" s="6" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="C53" s="6" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="D53" s="4" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="E53" s="2"/>
       <c r="F53" s="2"/>
@@ -3414,10 +3420,18 @@
       <c r="Y53" s="2"/>
     </row>
     <row r="54">
-      <c r="A54" s="2"/>
-      <c r="B54" s="2"/>
-      <c r="C54" s="2"/>
-      <c r="D54" s="2"/>
+      <c r="A54" s="3" t="s">
+        <v>129</v>
+      </c>
+      <c r="B54" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="C54" s="3" t="s">
+        <v>103</v>
+      </c>
+      <c r="D54" s="4" t="s">
+        <v>130</v>
+      </c>
       <c r="E54" s="2"/>
       <c r="F54" s="2"/>
       <c r="G54" s="2"/>
@@ -29020,8 +29034,9 @@
     <hyperlink r:id="rId61" ref="D52"/>
     <hyperlink r:id="rId62" ref="A53"/>
     <hyperlink r:id="rId63" ref="D53"/>
+    <hyperlink r:id="rId64" ref="D54"/>
   </hyperlinks>
-  <drawing r:id="rId64"/>
+  <drawing r:id="rId65"/>
 </worksheet>
 </file>
 
@@ -29040,10 +29055,10 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="8" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
       <c r="B1" s="8" t="s">
-        <v>129</v>
+        <v>132</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>1</v>
@@ -29078,7 +29093,7 @@
         <v>46</v>
       </c>
       <c r="B2" s="11" t="s">
-        <v>130</v>
+        <v>133</v>
       </c>
       <c r="C2" s="3" t="s">
         <v>46</v>
@@ -29111,7 +29126,7 @@
     <row r="3">
       <c r="A3" s="12"/>
       <c r="B3" s="13" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="C3" s="3" t="s">
         <v>46</v>
@@ -29144,7 +29159,7 @@
     <row r="4">
       <c r="A4" s="12"/>
       <c r="B4" s="11" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="C4" s="3" t="s">
         <v>46</v>
@@ -29177,7 +29192,7 @@
     <row r="5">
       <c r="A5" s="12"/>
       <c r="B5" s="11" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
       <c r="C5" s="3" t="s">
         <v>46</v>
@@ -29210,7 +29225,7 @@
     <row r="6">
       <c r="A6" s="12"/>
       <c r="B6" s="11" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="C6" s="3" t="s">
         <v>46</v>
@@ -29243,7 +29258,7 @@
     <row r="7">
       <c r="A7" s="12"/>
       <c r="B7" s="11" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="C7" s="3" t="s">
         <v>46</v>
@@ -29276,7 +29291,7 @@
     <row r="8">
       <c r="A8" s="12"/>
       <c r="B8" s="11" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="C8" s="3" t="s">
         <v>46</v>
@@ -29309,7 +29324,7 @@
     <row r="9">
       <c r="A9" s="12"/>
       <c r="B9" s="11" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="C9" s="3" t="s">
         <v>46</v>
@@ -29342,7 +29357,7 @@
     <row r="10">
       <c r="A10" s="12"/>
       <c r="B10" s="11" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
       <c r="C10" s="3" t="s">
         <v>46</v>
@@ -29375,7 +29390,7 @@
     <row r="11">
       <c r="A11" s="12"/>
       <c r="B11" s="11" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="C11" s="3" t="s">
         <v>46</v>
@@ -29408,7 +29423,7 @@
     <row r="12">
       <c r="A12" s="12"/>
       <c r="B12" s="11" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="C12" s="3" t="s">
         <v>46</v>
@@ -29441,7 +29456,7 @@
     <row r="13">
       <c r="A13" s="12"/>
       <c r="B13" s="13" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="C13" s="3" t="s">
         <v>46</v>
@@ -29474,7 +29489,7 @@
     <row r="14">
       <c r="A14" s="14"/>
       <c r="B14" s="11" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="C14" s="3" t="s">
         <v>46</v>
@@ -29506,10 +29521,10 @@
     </row>
     <row r="15">
       <c r="A15" s="10" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="B15" s="11" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="C15" s="3"/>
       <c r="D15" s="9"/>
@@ -29540,7 +29555,7 @@
     <row r="16">
       <c r="A16" s="14"/>
       <c r="B16" s="11" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="C16" s="3"/>
       <c r="D16" s="9"/>
@@ -29570,10 +29585,10 @@
     </row>
     <row r="17">
       <c r="A17" s="10" t="s">
-        <v>144</v>
+        <v>48</v>
       </c>
       <c r="B17" s="11" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="C17" s="3"/>
       <c r="D17" s="9"/>
@@ -29604,7 +29619,7 @@
     <row r="18">
       <c r="A18" s="12"/>
       <c r="B18" s="11" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="C18" s="3"/>
       <c r="D18" s="9"/>
@@ -29635,7 +29650,7 @@
     <row r="19">
       <c r="A19" s="12"/>
       <c r="B19" s="11" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="C19" s="3"/>
       <c r="D19" s="9"/>
@@ -29666,7 +29681,7 @@
     <row r="20">
       <c r="A20" s="12"/>
       <c r="B20" s="11" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="C20" s="3"/>
       <c r="D20" s="9"/>
@@ -29697,7 +29712,7 @@
     <row r="21">
       <c r="A21" s="12"/>
       <c r="B21" s="11" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="C21" s="3"/>
       <c r="D21" s="9"/>
@@ -29728,7 +29743,7 @@
     <row r="22">
       <c r="A22" s="14"/>
       <c r="B22" s="11" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="C22" s="3"/>
       <c r="D22" s="9"/>
@@ -29758,10 +29773,10 @@
     </row>
     <row r="23">
       <c r="A23" s="10" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="B23" s="11" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="C23" s="3"/>
       <c r="D23" s="9"/>
@@ -29792,7 +29807,7 @@
     <row r="24">
       <c r="A24" s="12"/>
       <c r="B24" s="11" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="D24" s="9"/>
       <c r="E24" s="9"/>
@@ -29822,7 +29837,7 @@
     <row r="25">
       <c r="A25" s="12"/>
       <c r="B25" s="11" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="D25" s="9"/>
       <c r="E25" s="9"/>
@@ -29852,7 +29867,7 @@
     <row r="26">
       <c r="A26" s="12"/>
       <c r="B26" s="11" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="C26" s="3"/>
       <c r="D26" s="9"/>
@@ -29883,7 +29898,7 @@
     <row r="27">
       <c r="A27" s="12"/>
       <c r="B27" s="11" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="D27" s="9"/>
       <c r="E27" s="9"/>
@@ -29913,7 +29928,7 @@
     <row r="28">
       <c r="A28" s="12"/>
       <c r="B28" s="11" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="D28" s="9"/>
       <c r="E28" s="9"/>
@@ -29943,7 +29958,7 @@
     <row r="29">
       <c r="A29" s="12"/>
       <c r="B29" s="11" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="C29" s="3"/>
       <c r="D29" s="9"/>
@@ -29974,7 +29989,7 @@
     <row r="30">
       <c r="A30" s="12"/>
       <c r="B30" s="11" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="D30" s="9"/>
       <c r="E30" s="9"/>
@@ -30004,7 +30019,7 @@
     <row r="31">
       <c r="A31" s="12"/>
       <c r="B31" s="11" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="D31" s="9"/>
       <c r="E31" s="9"/>
@@ -30034,7 +30049,7 @@
     <row r="32">
       <c r="A32" s="12"/>
       <c r="B32" s="11" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="D32" s="9"/>
       <c r="E32" s="9"/>
@@ -30064,7 +30079,7 @@
     <row r="33">
       <c r="A33" s="12"/>
       <c r="B33" s="11" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="D33" s="9"/>
       <c r="E33" s="9"/>
@@ -30094,7 +30109,7 @@
     <row r="34">
       <c r="A34" s="12"/>
       <c r="B34" s="11" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="D34" s="9"/>
       <c r="E34" s="9"/>
@@ -30124,7 +30139,7 @@
     <row r="35">
       <c r="A35" s="12"/>
       <c r="B35" s="11" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="D35" s="9"/>
       <c r="E35" s="9"/>
@@ -30154,7 +30169,7 @@
     <row r="36">
       <c r="A36" s="14"/>
       <c r="B36" s="11" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="D36" s="9"/>
       <c r="E36" s="9"/>
@@ -30183,10 +30198,10 @@
     </row>
     <row r="37">
       <c r="A37" s="10" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="B37" s="11" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="D37" s="9"/>
       <c r="E37" s="9"/>
@@ -30216,7 +30231,7 @@
     <row r="38">
       <c r="A38" s="12"/>
       <c r="B38" s="11" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="D38" s="9"/>
       <c r="E38" s="9"/>
@@ -30246,7 +30261,7 @@
     <row r="39">
       <c r="A39" s="12"/>
       <c r="B39" s="11" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="D39" s="9"/>
       <c r="E39" s="9"/>
@@ -30276,7 +30291,7 @@
     <row r="40">
       <c r="A40" s="12"/>
       <c r="B40" s="11" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="D40" s="9"/>
       <c r="E40" s="9"/>
@@ -30306,10 +30321,10 @@
     <row r="41">
       <c r="A41" s="12"/>
       <c r="B41" s="11" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="C41" s="6" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="D41" s="9"/>
       <c r="E41" s="9"/>
@@ -30339,7 +30354,7 @@
     <row r="42">
       <c r="A42" s="12"/>
       <c r="B42" s="11" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="C42" s="2"/>
       <c r="D42" s="9"/>
@@ -30370,7 +30385,7 @@
     <row r="43">
       <c r="A43" s="12"/>
       <c r="B43" s="11" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="C43" s="2"/>
       <c r="D43" s="9"/>
@@ -30401,7 +30416,7 @@
     <row r="44">
       <c r="A44" s="14"/>
       <c r="B44" s="11" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="C44" s="2"/>
       <c r="D44" s="9"/>
@@ -30431,10 +30446,10 @@
     </row>
     <row r="45">
       <c r="A45" s="10" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="B45" s="11" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="C45" s="2"/>
       <c r="D45" s="9"/>
@@ -30465,7 +30480,7 @@
     <row r="46">
       <c r="A46" s="12"/>
       <c r="B46" s="11" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="C46" s="2"/>
       <c r="D46" s="9"/>
@@ -30496,7 +30511,7 @@
     <row r="47">
       <c r="A47" s="12"/>
       <c r="B47" s="11" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="C47" s="2"/>
       <c r="D47" s="9"/>
@@ -30527,7 +30542,7 @@
     <row r="48">
       <c r="A48" s="12"/>
       <c r="B48" s="11" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="C48" s="2"/>
       <c r="D48" s="9"/>
@@ -30558,7 +30573,7 @@
     <row r="49">
       <c r="A49" s="12"/>
       <c r="B49" s="11" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="C49" s="2"/>
       <c r="D49" s="9"/>
@@ -30589,7 +30604,7 @@
     <row r="50">
       <c r="A50" s="14"/>
       <c r="B50" s="11" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="C50" s="2"/>
       <c r="D50" s="9"/>
@@ -30619,10 +30634,10 @@
     </row>
     <row r="51">
       <c r="A51" s="10" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="B51" s="11" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="C51" s="2"/>
       <c r="D51" s="9"/>
@@ -30653,7 +30668,7 @@
     <row r="52">
       <c r="A52" s="12"/>
       <c r="B52" s="11" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="C52" s="2"/>
       <c r="D52" s="9"/>
@@ -30684,7 +30699,7 @@
     <row r="53">
       <c r="A53" s="14"/>
       <c r="B53" s="11" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="C53" s="2"/>
       <c r="D53" s="9"/>

</xml_diff>